<commit_message>
Added Washington DC Resources
</commit_message>
<xml_diff>
--- a/public/Autism_Resources_by_State.xlsx
+++ b/public/Autism_Resources_by_State.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\Spectrum Works Projects\autism_resources_by_state\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B4EB5C-DD61-4D68-8DA1-0D332E0D5685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8389165D-C633-4E5D-BEAF-F21124FB39AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3168" yWindow="264" windowWidth="13284" windowHeight="13416" xr2:uid="{BB264F5C-C314-4413-9F4B-48BA520C8538}"/>
+    <workbookView xWindow="10608" yWindow="1164" windowWidth="13284" windowHeight="13416" xr2:uid="{BB264F5C-C314-4413-9F4B-48BA520C8538}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="516">
   <si>
     <t>Resource</t>
   </si>
@@ -1559,6 +1559,33 @@
   </si>
   <si>
     <t>Association for Autism and Neurodiversity (AANE)</t>
+  </si>
+  <si>
+    <t>Washington DC</t>
+  </si>
+  <si>
+    <t>https://www.childrensnational.org/get-care/departments/center-for-autism-spectrum-disorders</t>
+  </si>
+  <si>
+    <t>Center for Autism Spectrum Disorders</t>
+  </si>
+  <si>
+    <t>https://www.dcautismparents.org/</t>
+  </si>
+  <si>
+    <t>DC Autism Parents</t>
+  </si>
+  <si>
+    <t>https://www.childrensnational.org/in-the-community/advocacy-and-outreach/community-initiatives-and-partnerships/dc-autism-collaborative</t>
+  </si>
+  <si>
+    <t>DC Autism Collaborative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JSSA </t>
+  </si>
+  <si>
+    <t>https://www.jssa.org/services/disability-employment/</t>
   </si>
 </sst>
 </file>
@@ -1603,10 +1630,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1630,8 +1659,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{34C68183-241C-4606-AC66-490183F44371}" name="Table1" displayName="Table1" ref="A1:E272" totalsRowShown="0" dataCellStyle="Normal">
-  <autoFilter ref="A1:E272" xr:uid="{34C68183-241C-4606-AC66-490183F44371}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{34C68183-241C-4606-AC66-490183F44371}" name="Table1" displayName="Table1" ref="A1:E277" totalsRowShown="0" dataCellStyle="Normal">
+  <autoFilter ref="A1:E277" xr:uid="{34C68183-241C-4606-AC66-490183F44371}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E272">
     <sortCondition descending="1" ref="D1:D272"/>
   </sortState>
@@ -1965,7 +1994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F8DAF23-311A-4B42-861B-1D5FBACA69D7}">
-  <dimension ref="A1:E272"/>
+  <dimension ref="A1:E277"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.77734375" customWidth="1"/>
@@ -6349,6 +6378,86 @@
         <v>13</v>
       </c>
       <c r="E272" t="b">
+        <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A273" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D273" s="3"/>
+      <c r="E273" s="4" t="b">
+        <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A274" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D274" s="3"/>
+      <c r="E274" s="4" t="b">
+        <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A275" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="B275" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D275" s="3"/>
+      <c r="E275" s="4" t="b">
+        <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A276" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D276" s="3"/>
+      <c r="E276" s="4" t="b">
+        <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A277" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="B277" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D277" s="3"/>
+      <c r="E277" s="4" t="b">
         <f>IF(ISNUMBER(SEARCH("gov",Table1[[#This Row],[Link]])),TRUE,FALSE)</f>
         <v>0</v>
       </c>
@@ -6443,11 +6552,12 @@
     <hyperlink ref="B95" r:id="rId86" xr:uid="{0E5CF849-68AF-473C-924A-E50CF4FD5146}"/>
     <hyperlink ref="B44" r:id="rId87" xr:uid="{4EB66C43-78F9-4894-8EDA-FC133DB819F0}"/>
     <hyperlink ref="B96" r:id="rId88" xr:uid="{D19E63AE-3F40-4E59-BC44-086BE15C629D}"/>
+    <hyperlink ref="B277" r:id="rId89" xr:uid="{CF1B6DAB-9D58-4E89-B897-CE509CC7C5FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId89"/>
+  <pageSetup orientation="portrait" r:id="rId90"/>
   <tableParts count="1">
-    <tablePart r:id="rId90"/>
+    <tablePart r:id="rId91"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>